<commit_message>
feat: rediseña las actividades con casos prácticos y nuevos archivos de datos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/datos/1.4_Formulas_basicas.xlsx
+++ b/public/datos/1.4_Formulas_basicas.xlsx
@@ -7,9 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Horas_Documentacion" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Parametros" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Presupuesto_SIG" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,10 +60,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,112 +437,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="37" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Código</t>
+          <t>Parámetro</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Documento</t>
+          <t>Valor</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Proceso</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Horas de elaboración</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Costo</t>
+          <t>Instrucciones de la Actividad</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PE-01-PO-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Política del SIG</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Direccionamiento estratégico</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>14</v>
+          <t>Tarifa fija por hora ($)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>28500</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>1. En la columna 'Costo ($)' calcula =Horas * $B$2 (fijando B2 con $). 2. Completa el resumen al final con SUMA, PROMEDIO y CONTAR.</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>PE-01-PL-01</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Plan estratégico 2025-2028</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Direccionamiento estratégico</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>16</v>
-      </c>
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PE-01-PR-01</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Revisión por la dirección</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Direccionamiento estratégico</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>8</v>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Documento</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Proceso</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Horas de elaboración</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Costo ($)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PE-01-FO-01</t>
+          <t>PE-01-PO-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Acta de revisión por la dirección</t>
+          <t>Política del SIG</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -547,72 +536,72 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PE-02-MA-01</t>
+          <t>PE-01-PL-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Manual del SIG</t>
+          <t>Plan estratégico 2025-2028</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gestión de la calidad</t>
+          <t>Direccionamiento estratégico</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PE-02-PR-01</t>
+          <t>PE-01-PR-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Control de documentos</t>
+          <t>Revisión por la dirección</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gestión de la calidad</t>
+          <t>Direccionamiento estratégico</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PE-02-PR-02</t>
+          <t>PE-01-FO-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Auditorías internas</t>
+          <t>Acta de revisión por la dirección</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gestión de la calidad</t>
+          <t>Direccionamiento estratégico</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PE-02-PR-03</t>
+          <t>PE-02-MA-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Acciones correctivas</t>
+          <t>Manual del SIG</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -621,18 +610,18 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PE-02-FO-01</t>
+          <t>PE-02-PR-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Listado maestro de documentos</t>
+          <t>Control de documentos</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -641,18 +630,18 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PE-02-FO-02</t>
+          <t>PE-02-PR-02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Plan de auditoría</t>
+          <t>Auditorías internas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -661,78 +650,78 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PM-01-PR-01</t>
+          <t>PE-02-PR-03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Control de producción</t>
+          <t>Acciones correctivas</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Producción</t>
+          <t>Gestión de la calidad</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PM-01-IN-01</t>
+          <t>PE-02-FO-01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Limpieza y desinfección de equipos</t>
+          <t>Listado maestro de documentos</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Producción</t>
+          <t>Gestión de la calidad</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PM-01-IN-02</t>
+          <t>PE-02-FO-02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pasteurización</t>
+          <t>Plan de auditoría</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Producción</t>
+          <t>Gestión de la calidad</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PM-01-FO-01</t>
+          <t>PM-01-PR-01</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Registro de temperatura</t>
+          <t>Control de producción</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -741,128 +730,137 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>PM-01-IN-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Limpieza y desinfección de equipos</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PM-01-IN-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pasteurización</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PM-01-FO-01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Registro de temperatura</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>PM-01-FO-02</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Control de lotes</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Producción</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D19" t="n">
         <v>12</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Total de horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Promedio de horas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Costo total liquidado</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Cantidad de documentos</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Parámetro</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Valor hora de elaboración</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>28500</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Medida</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Resultado</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Total de horas</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Promedio de horas por documento</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cantidad de documentos</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Costo total</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="C1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>